<commit_message>
refactor: 將 display_order 重新命名為 display_order_id
</commit_message>
<xml_diff>
--- a/excel-data/restaurant.xlsx
+++ b/excel-data/restaurant.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyCreation\Web\mogumogu-pick\excel-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0030A1-C291-4125-AC00-F375C5E691D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCBCBB03-6D46-4202-8945-50FA3121ECAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2C4057A3-4DF4-41B5-A441-0D94A14DFD1E}"/>
+    <workbookView xWindow="1164" yWindow="2592" windowWidth="17280" windowHeight="9648" xr2:uid="{2C4057A3-4DF4-41B5-A441-0D94A14DFD1E}"/>
   </bookViews>
   <sheets>
     <sheet name="restaurant" sheetId="1" r:id="rId1"/>
@@ -606,14 +606,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>群組內排序</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>display_order</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>selected_count</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -647,6 +639,14 @@
   </si>
   <si>
     <t>is_archived</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>display_order_id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>群組內排序 ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1100,10 +1100,10 @@
         <v>183</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>160</v>
@@ -1115,16 +1115,16 @@
         <v>161</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J1" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>191</v>
-      </c>
       <c r="L1" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -1138,10 +1138,10 @@
         <v>184</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>1</v>
@@ -1153,16 +1153,16 @@
         <v>2</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>